<commit_message>
- archive stale files - add fulltext screening reviewer decision
</commit_message>
<xml_diff>
--- a/slr_artifacts/20260609_095939_tunneling-jellyfish-of-fascination/4_Fulltext_Screening/Reviewer_Decision_Fulltext_Screening.xlsx
+++ b/slr_artifacts/20260609_095939_tunneling-jellyfish-of-fascination/4_Fulltext_Screening/Reviewer_Decision_Fulltext_Screening.xlsx
@@ -5,18 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rreider\Nextcloud3\PhD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ladmin\PycharmProjects\slr-artifacts\slr_artifacts\20260609_095939_tunneling-jellyfish-of-fascination\4_Fulltext_Screening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8FF8285-051A-494C-A3BA-39701E595F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF4CC49-3524-4B8B-A2D9-109311CBF35A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7B1B9799-EF01-4970-ADB2-A4164EBCB5ED}"/>
+    <workbookView xWindow="6825" yWindow="2430" windowWidth="28800" windowHeight="14595" xr2:uid="{7B1B9799-EF01-4970-ADB2-A4164EBCB5ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$17</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -193,9 +195,6 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>Investigate</t>
-  </si>
-  <si>
     <t>Investigate (pass ok from R2)</t>
   </si>
   <si>
@@ -215,6 +214,9 @@
   </si>
   <si>
     <t>R1 Investigation: The paper considers a facility location problem scenario as one of its 5 scenarios, which is a strategic and system configuring planning problem</t>
+  </si>
+  <si>
+    <t>Pass after discussion</t>
   </si>
 </sst>
 </file>
@@ -300,28 +302,28 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -651,122 +653,122 @@
       <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6" t="s">
+      <c r="G1" s="13"/>
+      <c r="H1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6" t="s">
+      <c r="I1" s="13"/>
+      <c r="J1" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6" t="s">
+      <c r="K1" s="13"/>
+      <c r="L1" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6" t="s">
+      <c r="M1" s="13"/>
+      <c r="N1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6" t="s">
+      <c r="O1" s="13"/>
+      <c r="P1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6" t="s">
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6" t="s">
+      <c r="S1" s="13"/>
+      <c r="T1" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="U1" s="6"/>
-      <c r="V1" s="6" t="s">
+      <c r="U1" s="13"/>
+      <c r="V1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="W1" s="6"/>
-      <c r="X1" s="6" t="s">
+      <c r="W1" s="13"/>
+      <c r="X1" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="Y1" s="6"/>
-      <c r="Z1" s="6" t="s">
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="AA1" s="6"/>
-      <c r="AB1" s="6" t="s">
+      <c r="AA1" s="13"/>
+      <c r="AB1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="AC1" s="6"/>
-      <c r="AD1" s="6" t="s">
+      <c r="AC1" s="13"/>
+      <c r="AD1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="AE1" s="6"/>
-      <c r="AF1" s="6" t="s">
+      <c r="AE1" s="13"/>
+      <c r="AF1" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="AG1" s="6"/>
-      <c r="AH1" s="6" t="s">
+      <c r="AG1" s="13"/>
+      <c r="AH1" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="AI1" s="6"/>
-      <c r="AJ1" s="6" t="s">
+      <c r="AI1" s="13"/>
+      <c r="AJ1" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="AK1" s="6"/>
-      <c r="AL1" s="6" t="s">
+      <c r="AK1" s="13"/>
+      <c r="AL1" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="AM1" s="6"/>
-      <c r="AN1" s="8" t="s">
+      <c r="AM1" s="13"/>
+      <c r="AN1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="AO1" s="8"/>
-      <c r="AP1" s="6" t="s">
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="AQ1" s="6"/>
-      <c r="AR1" s="6" t="s">
+      <c r="AQ1" s="13"/>
+      <c r="AR1" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="AS1" s="6"/>
-      <c r="AT1" s="6" t="s">
+      <c r="AS1" s="13"/>
+      <c r="AT1" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="AU1" s="6"/>
-      <c r="AV1" s="6" t="s">
+      <c r="AU1" s="13"/>
+      <c r="AV1" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="AW1" s="6"/>
-      <c r="AX1" s="6" t="s">
+      <c r="AW1" s="13"/>
+      <c r="AX1" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="AY1" s="6"/>
-      <c r="AZ1" s="6" t="s">
+      <c r="AY1" s="13"/>
+      <c r="AZ1" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="BA1" s="6"/>
-      <c r="BB1" s="6" t="s">
+      <c r="BA1" s="13"/>
+      <c r="BB1" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="BC1" s="6"/>
-      <c r="BD1" s="6" t="s">
+      <c r="BC1" s="13"/>
+      <c r="BD1" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="BE1" s="6"/>
-      <c r="BF1" s="6" t="s">
+      <c r="BE1" s="13"/>
+      <c r="BF1" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="BG1" s="6"/>
+      <c r="BG1" s="13"/>
     </row>
     <row r="2" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1113,13 +1115,13 @@
       <c r="BC3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD3" s="10" t="s">
+      <c r="BD3" s="12" t="s">
         <v>47</v>
       </c>
       <c r="BE3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF3" s="10" t="s">
+      <c r="BF3" s="12" t="s">
         <v>47</v>
       </c>
       <c r="BG3" s="4" t="s">
@@ -1292,11 +1294,11 @@
       <c r="BC4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD4" s="10"/>
+      <c r="BD4" s="12"/>
       <c r="BE4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF4" s="10"/>
+      <c r="BF4" s="12"/>
       <c r="BG4" s="4" t="s">
         <v>7</v>
       </c>
@@ -1467,11 +1469,11 @@
       <c r="BC5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD5" s="10"/>
+      <c r="BD5" s="12"/>
       <c r="BE5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF5" s="10"/>
+      <c r="BF5" s="12"/>
       <c r="BG5" s="4" t="s">
         <v>7</v>
       </c>
@@ -1642,11 +1644,11 @@
       <c r="BC6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD6" s="10"/>
+      <c r="BD6" s="12"/>
       <c r="BE6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF6" s="10"/>
+      <c r="BF6" s="12"/>
       <c r="BG6" s="4" t="s">
         <v>7</v>
       </c>
@@ -1817,11 +1819,11 @@
       <c r="BC7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD7" s="10"/>
+      <c r="BD7" s="12"/>
       <c r="BE7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF7" s="10"/>
+      <c r="BF7" s="12"/>
       <c r="BG7" s="4" t="s">
         <v>7</v>
       </c>
@@ -1992,11 +1994,11 @@
       <c r="BC8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD8" s="10"/>
+      <c r="BD8" s="12"/>
       <c r="BE8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF8" s="10"/>
+      <c r="BF8" s="12"/>
       <c r="BG8" s="4" t="s">
         <v>7</v>
       </c>
@@ -2167,11 +2169,11 @@
       <c r="BC9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD9" s="10"/>
+      <c r="BD9" s="12"/>
       <c r="BE9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF9" s="10"/>
+      <c r="BF9" s="12"/>
       <c r="BG9" s="4" t="s">
         <v>7</v>
       </c>
@@ -2342,11 +2344,11 @@
       <c r="BC10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD10" s="10"/>
+      <c r="BD10" s="12"/>
       <c r="BE10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF10" s="10"/>
+      <c r="BF10" s="12"/>
       <c r="BG10" s="4" t="s">
         <v>7</v>
       </c>
@@ -2517,11 +2519,11 @@
       <c r="BC11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD11" s="10"/>
+      <c r="BD11" s="12"/>
       <c r="BE11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF11" s="10"/>
+      <c r="BF11" s="12"/>
       <c r="BG11" s="4" t="s">
         <v>7</v>
       </c>
@@ -2692,11 +2694,11 @@
       <c r="BC12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD12" s="10"/>
+      <c r="BD12" s="12"/>
       <c r="BE12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF12" s="10"/>
+      <c r="BF12" s="12"/>
       <c r="BG12" s="4" t="s">
         <v>7</v>
       </c>
@@ -2867,11 +2869,11 @@
       <c r="BC13" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD13" s="10"/>
+      <c r="BD13" s="12"/>
       <c r="BE13" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF13" s="10"/>
+      <c r="BF13" s="12"/>
       <c r="BG13" s="4" t="s">
         <v>7</v>
       </c>
@@ -3042,164 +3044,215 @@
       <c r="BC14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BD14" s="10"/>
+      <c r="BD14" s="12"/>
       <c r="BE14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="BF14" s="10"/>
+      <c r="BF14" s="12"/>
       <c r="BG14" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:59" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:59" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13" t="s">
+      <c r="C16" s="11"/>
+      <c r="D16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13" t="s">
+      <c r="E16" s="11"/>
+      <c r="F16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13" t="s">
+      <c r="G16" s="11"/>
+      <c r="H16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="I16" s="13"/>
-      <c r="J16" s="14" t="s">
+      <c r="I16" s="11"/>
+      <c r="J16" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="K16" s="14"/>
-      <c r="L16" s="13" t="s">
+      <c r="K16" s="9"/>
+      <c r="L16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13" t="s">
+      <c r="M16" s="11"/>
+      <c r="N16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="O16" s="13"/>
-      <c r="P16" s="14" t="s">
+      <c r="O16" s="11"/>
+      <c r="P16" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="Q16" s="14"/>
-      <c r="R16" s="11" t="s">
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="U16" s="9"/>
+      <c r="V16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="W16" s="9"/>
+      <c r="X16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y16" s="11"/>
+      <c r="Z16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA16" s="11"/>
+      <c r="AB16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC16" s="11"/>
+      <c r="AD16" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="S16" s="11"/>
-      <c r="T16" s="11" t="s">
+      <c r="AE16" s="9"/>
+      <c r="AF16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AG16" s="11"/>
+      <c r="AH16" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI16" s="11"/>
+      <c r="AJ16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AK16" s="11"/>
+      <c r="AL16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM16" s="11"/>
+      <c r="AN16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO16" s="11"/>
+      <c r="AP16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ16" s="9"/>
+      <c r="AR16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AS16" s="11"/>
+      <c r="AT16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU16" s="9"/>
+      <c r="AV16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AW16" s="9"/>
+      <c r="AX16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY16" s="11"/>
+      <c r="AZ16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="BA16" s="11"/>
+      <c r="BB16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="BC16" s="9"/>
+      <c r="BD16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="BE16" s="9"/>
+      <c r="BF16" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="BG16" s="9"/>
+    </row>
+    <row r="17" spans="18:49" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R17" s="14"/>
+      <c r="S17" s="14"/>
+      <c r="T17" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="U16" s="11"/>
-      <c r="V16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="W16" s="14"/>
-      <c r="X16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="Y16" s="13"/>
-      <c r="Z16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA16" s="13"/>
-      <c r="AB16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AC16" s="13"/>
-      <c r="AD16" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE16" s="11"/>
-      <c r="AF16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG16" s="13"/>
-      <c r="AH16" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="AI16" s="13"/>
-      <c r="AJ16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AK16" s="13"/>
-      <c r="AL16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AM16" s="13"/>
-      <c r="AN16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AO16" s="13"/>
-      <c r="AP16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="AQ16" s="14"/>
-      <c r="AR16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AS16" s="13"/>
-      <c r="AT16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="AU16" s="14"/>
-      <c r="AV16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW16" s="14"/>
-      <c r="AX16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AY16" s="13"/>
-      <c r="AZ16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="BA16" s="13"/>
-      <c r="BB16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="BC16" s="14"/>
-      <c r="BD16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="BE16" s="14"/>
-      <c r="BF16" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="BG16" s="14"/>
-    </row>
-    <row r="17" spans="20:49" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="T17" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="U17" s="8"/>
+      <c r="U17" s="10"/>
       <c r="AC17" s="3"/>
-      <c r="AD17" s="7" t="s">
-        <v>58</v>
+      <c r="AD17" s="6" t="s">
+        <v>57</v>
       </c>
       <c r="AE17" s="3"/>
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
-      <c r="AH17" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="AI17" s="8"/>
+      <c r="AH17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI17" s="10"/>
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
       <c r="AL17" s="3"/>
       <c r="AM17" s="3"/>
       <c r="AN17" s="3"/>
-      <c r="AV17" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AW17" s="8"/>
+      <c r="AV17" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW17" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="63">
+  <autoFilter ref="A1:A17" xr:uid="{D87C004D-8D13-44A6-A3B7-B98154F09A59}"/>
+  <mergeCells count="64">
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="AB1:AC1"/>
+    <mergeCell ref="AD1:AE1"/>
+    <mergeCell ref="AF1:AG1"/>
+    <mergeCell ref="AH1:AI1"/>
+    <mergeCell ref="AJ1:AK1"/>
+    <mergeCell ref="AZ1:BA1"/>
+    <mergeCell ref="BB1:BC1"/>
+    <mergeCell ref="BD1:BE1"/>
+    <mergeCell ref="AL1:AM1"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AR1:AS1"/>
+    <mergeCell ref="AT1:AU1"/>
+    <mergeCell ref="BF1:BG1"/>
+    <mergeCell ref="BF3:BF14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="V16:W16"/>
+    <mergeCell ref="X16:Y16"/>
+    <mergeCell ref="AV1:AW1"/>
+    <mergeCell ref="AX1:AY1"/>
+    <mergeCell ref="AB16:AC16"/>
+    <mergeCell ref="AD16:AE16"/>
+    <mergeCell ref="AF16:AG16"/>
+    <mergeCell ref="AH16:AI16"/>
+    <mergeCell ref="BD3:BD14"/>
     <mergeCell ref="BD16:BE16"/>
     <mergeCell ref="BF16:BG16"/>
     <mergeCell ref="T17:U17"/>
@@ -3216,53 +3269,6 @@
     <mergeCell ref="AP16:AQ16"/>
     <mergeCell ref="AR16:AS16"/>
     <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="AB16:AC16"/>
-    <mergeCell ref="AD16:AE16"/>
-    <mergeCell ref="AF16:AG16"/>
-    <mergeCell ref="AH16:AI16"/>
-    <mergeCell ref="BD3:BD14"/>
-    <mergeCell ref="BF1:BG1"/>
-    <mergeCell ref="BF3:BF14"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="T16:U16"/>
-    <mergeCell ref="V16:W16"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="AV1:AW1"/>
-    <mergeCell ref="AX1:AY1"/>
-    <mergeCell ref="AZ1:BA1"/>
-    <mergeCell ref="BB1:BC1"/>
-    <mergeCell ref="BD1:BE1"/>
-    <mergeCell ref="AL1:AM1"/>
-    <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AP1:AQ1"/>
-    <mergeCell ref="AR1:AS1"/>
-    <mergeCell ref="AT1:AU1"/>
-    <mergeCell ref="AB1:AC1"/>
-    <mergeCell ref="AD1:AE1"/>
-    <mergeCell ref="AF1:AG1"/>
-    <mergeCell ref="AH1:AI1"/>
-    <mergeCell ref="AJ1:AK1"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>